<commit_message>
Update iKS 2026-2q questionnaire: fix company identity, drop comment note
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181ApW5pLdnzCkrJhMjpBJs
</commit_message>
<xml_diff>
--- a/Анкета iKS_Consulting_clouds_2026-2q_ИТОГ.xlsx
+++ b/Анкета iKS_Consulting_clouds_2026-2q_ИТОГ.xlsx
@@ -2211,11 +2211,11 @@
     <col width="6.59765625" customWidth="1" min="21" max="25"/>
     <col width="6.19921875" customWidth="1" min="26" max="26"/>
     <col width="1.59765625" customWidth="1" min="27" max="27"/>
-    <col hidden="1" style="30" min="28" max="34"/>
+    <col hidden="1" width="13" customWidth="1" style="30" min="28" max="34"/>
     <col hidden="1" width="8.796875" customWidth="1" style="30" min="35" max="35"/>
-    <col hidden="1" style="30" min="36" max="42"/>
+    <col hidden="1" width="13" customWidth="1" style="30" min="36" max="42"/>
     <col hidden="1" width="8.796875" customWidth="1" style="30" min="43" max="43"/>
-    <col hidden="1" style="30" min="44" max="61"/>
+    <col hidden="1" width="13" customWidth="1" style="30" min="44" max="61"/>
     <col hidden="1" width="5" customWidth="1" style="30" min="62" max="16384"/>
   </cols>
   <sheetData>
@@ -2326,7 +2326,7 @@
       <c r="D4" s="137" t="n"/>
       <c r="E4" s="116" t="inlineStr">
         <is>
-          <t>ООО "Флекс"</t>
+          <t>ООО «БЕАР-СОФТ»</t>
         </is>
       </c>
       <c r="F4" s="138" t="n"/>
@@ -2392,7 +2392,7 @@
       <c r="D6" s="137" t="n"/>
       <c r="E6" s="116" t="inlineStr">
         <is>
-          <t>Cloud4Y</t>
+          <t>Cloud4U</t>
         </is>
       </c>
       <c r="F6" s="138" t="n"/>
@@ -12173,11 +12173,7 @@
       <c r="K223" s="144" t="n"/>
     </row>
     <row r="224" ht="25.5" customFormat="1" customHeight="1" s="19">
-      <c r="B224" s="130" t="inlineStr">
-        <is>
-          <t>Автозаполнение на базе анкеты 2025-4q. Столбец 2025 (итог) перенесён из итогов 2025. Кварталы 2026 = годовой прогноз компании (2026), распределённый по квартальной сезонности 2025 из прошлой анкеты (доли 21/25/26/27%). Bare Metal 2025 разбит на без/с GPU в пропорции прогноза 2026. Таблицы 9,11,12,13,14 и кол-во клиентов данных не имели ни в одной анкете — оставлены пустыми.</t>
-        </is>
-      </c>
+      <c r="B224" s="130" t="n"/>
       <c r="C224" s="159" t="n"/>
       <c r="D224" s="159" t="n"/>
       <c r="E224" s="159" t="n"/>

</xml_diff>